<commit_message>
Legislative Studies Quarterly: note the separate title page and short-form limits
The 10,000-word limit is unchanged and still undefined as to what counts; the
entry now says so plainly, and notes the double-anonymized title page, the
150-word abstract and the 100-word author biography.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Political_Science_Journal_Word_Limits.xlsx
+++ b/data/source/Political_Science_Journal_Word_Limits.xlsx
@@ -2498,12 +2498,12 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>No detailed included/excluded component definition found.</t>
+          <t>The guidelines ask for the manuscript's word count, not exceeding 10,000 words, but do not say which parts count.</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Research articles.</t>
+          <t>Research articles; rechecked 16 October 2026. Review is double-anonymized, so the title page, which carries the word count and an author biography of up to 100 words, is a separate file. Abstract suggested at 150 words or fewer.</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">

</xml_diff>